<commit_message>
fix: cotización monotributo usa Plan Joven y aportes actualizados (MAYO 2026); bootstrap re-importa precios/aportes en cada deploy
</commit_message>
<xml_diff>
--- a/servired_knowledge/aportes/aportes_monotributo.xlsx
+++ b/servired_knowledge/aportes/aportes_monotributo.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Aportes Monotributo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aportes Monotributo" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -435,7 +435,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5386.79</v>
+        <v>19791.1</v>
       </c>
     </row>
     <row r="3">
@@ -445,7 +445,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8002.16</v>
+        <v>19791.1</v>
       </c>
     </row>
     <row r="4">
@@ -455,7 +455,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10619.24</v>
+        <v>19791.1</v>
       </c>
     </row>
     <row r="5">
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>14423.55</v>
+        <v>23519.86</v>
       </c>
     </row>
     <row r="6">
@@ -475,7 +475,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>19161.57</v>
+        <v>28682.75</v>
       </c>
     </row>
     <row r="7">
@@ -485,7 +485,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>24595.82</v>
+        <v>32985.17</v>
       </c>
     </row>
     <row r="8">
@@ -495,7 +495,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>30030.08</v>
+        <v>35566.62</v>
       </c>
     </row>
     <row r="9">
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>49057.49</v>
+        <v>52776.27</v>
       </c>
     </row>
     <row r="11">
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>55546.67</v>
+        <v>59229.89</v>
       </c>
     </row>
     <row r="12">
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>62918.02</v>
+        <v>67691.31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>